<commit_message>
Add Streamlit web app
</commit_message>
<xml_diff>
--- a/File1.xlsx
+++ b/File1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EmailsWorkTranslator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ACDDA9F-F605-44A5-B277-2194C96A38C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D4C72C-0929-43AB-B32E-120069D10F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{8CB61D00-9AB9-4E83-BD42-C3B4D184A08F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{8CB61D00-9AB9-4E83-BD42-C3B4D184A08F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="500">
   <si>
     <t>البريد الالكترونى</t>
   </si>
@@ -1519,6 +1519,12 @@
   </si>
   <si>
     <t>Mohmd AbdAlzym Ebrahym Aldswqy</t>
+  </si>
+  <si>
+    <t>الاسم باللغة الانجليزية</t>
+  </si>
+  <si>
+    <t>الاسم</t>
   </si>
 </sst>
 </file>
@@ -1578,9 +1584,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1618,7 +1624,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1724,7 +1730,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1866,7 +1872,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1887,6 +1893,12 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="C1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D1" t="s">
+        <v>498</v>
+      </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">

</xml_diff>